<commit_message>
revise ind names for older children
</commit_message>
<xml_diff>
--- a/www/Upload_ISO3Code_example_single_region.xlsx
+++ b/www/Upload_ISO3Code_example_single_region.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyhel\Dropbox\UNICEF_Work_Project\191011_Shiny_regional_aggregate\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBE0A377-89BE-4D3B-9339-1F0A89E2445F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD41DD3F-53BD-49A8-BE10-3D5E41AB5183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
     <t>Afghanistan</t>
   </si>
   <si>
-    <t>WB Low income countries</t>
-  </si>
-  <si>
     <t>BDI</t>
   </si>
   <si>
@@ -212,6 +209,9 @@
   </si>
   <si>
     <t>5. This example list will produce the aggregates for the 27 low-income countries (one of the World Bank region)</t>
+  </si>
+  <si>
+    <t>Low income countries</t>
   </si>
 </sst>
 </file>
@@ -1097,7 +1097,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1108,308 +1108,308 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
         <v>24</v>
       </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
-        <v>27</v>
-      </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
         <v>28</v>
       </c>
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
       <c r="C14" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
         <v>32</v>
       </c>
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
       <c r="C16" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" t="s">
         <v>34</v>
       </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
       <c r="C17" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
         <v>36</v>
       </c>
-      <c r="B18" t="s">
-        <v>37</v>
-      </c>
       <c r="C18" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" t="s">
         <v>38</v>
       </c>
-      <c r="B19" t="s">
-        <v>39</v>
-      </c>
       <c r="C19" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" t="s">
         <v>40</v>
       </c>
-      <c r="B20" t="s">
-        <v>41</v>
-      </c>
       <c r="C20" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" t="s">
         <v>42</v>
       </c>
-      <c r="B21" t="s">
-        <v>43</v>
-      </c>
       <c r="C21" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" t="s">
         <v>44</v>
       </c>
-      <c r="B22" t="s">
-        <v>45</v>
-      </c>
       <c r="C22" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" t="s">
         <v>46</v>
       </c>
-      <c r="B23" t="s">
-        <v>47</v>
-      </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
         <v>48</v>
       </c>
-      <c r="B24" t="s">
-        <v>49</v>
-      </c>
       <c r="C24" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
         <v>50</v>
       </c>
-      <c r="B25" t="s">
-        <v>51</v>
-      </c>
       <c r="C25" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
         <v>52</v>
       </c>
-      <c r="B26" t="s">
-        <v>53</v>
-      </c>
       <c r="C26" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" t="s">
         <v>54</v>
       </c>
-      <c r="B27" t="s">
-        <v>55</v>
-      </c>
       <c r="C27" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
         <v>56</v>
       </c>
-      <c r="B28" t="s">
-        <v>57</v>
-      </c>
       <c r="C28" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update to IGME 2022
</commit_message>
<xml_diff>
--- a/www/Upload_ISO3Code_example_single_region.xlsx
+++ b/www/Upload_ISO3Code_example_single_region.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyhel\Dropbox\UNICEF_Work_Project\191011_Shiny_regional_aggregate\www\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyhel\Dropbox\UNICEF Work\Revision.Shiny\Shiny2022\Shiny_regional_aggregate\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD41DD3F-53BD-49A8-BE10-3D5E41AB5183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98BF411-BB8C-4B7A-9226-524573D1A772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Upload_ISO3Code_example_single_" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="66">
   <si>
     <t>ISO3Code</t>
   </si>
@@ -212,6 +212,12 @@
   </si>
   <si>
     <t>Low income countries</t>
+  </si>
+  <si>
+    <t>ZMB</t>
+  </si>
+  <si>
+    <t>Zambia</t>
   </si>
 </sst>
 </file>
@@ -1070,7 +1076,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1078,7 +1084,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1130,10 +1136,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
         <v>63</v>
@@ -1144,10 +1150,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
         <v>63</v>
@@ -1172,10 +1178,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>63</v>
@@ -1183,10 +1189,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
         <v>63</v>
@@ -1194,10 +1200,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
         <v>63</v>
@@ -1205,10 +1211,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
         <v>63</v>
@@ -1216,10 +1222,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
         <v>63</v>
@@ -1249,10 +1255,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
         <v>63</v>
@@ -1260,10 +1266,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
         <v>63</v>
@@ -1271,10 +1277,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
         <v>63</v>
@@ -1293,10 +1299,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
         <v>63</v>
@@ -1315,10 +1321,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
         <v>63</v>
@@ -1326,10 +1332,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
         <v>63</v>
@@ -1337,10 +1343,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C22" t="s">
         <v>63</v>
@@ -1348,10 +1354,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
         <v>63</v>
@@ -1370,10 +1376,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1381,10 +1387,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C26" t="s">
         <v>63</v>
@@ -1392,10 +1398,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="C27" t="s">
         <v>63</v>
@@ -1409,6 +1415,17 @@
         <v>56</v>
       </c>
       <c r="C28" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>